<commit_message>
Let the client tick placements instead of unticking them
The wizard's result list arrived with every placement pre-checked, so the
client's job was to remove what they did not want. That is backwards for a
suggestion list. Boxes start empty, a counter shows what is selected and what
it costs, and one button ticks or clears the whole list for the case where
they do want everything.

Checked the address programme against the customer's file line by line: 52
addresses and 270 positions, matching. One name on the site carried a suffix
the file does not have — "ул. Кирова, 12 (ЛиЛия)" is now "ул. Кирова, 12" —
and the designer's sheet is rebuilt with it.

A side with a single position was described as "один раз за оборот из 1". It
now says the poster is visible the whole time, which is what one position means.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Фото_площадок_задание_дизайнеру.xlsx
+++ b/Фото_площадок_задание_дизайнеру.xlsx
@@ -1159,7 +1159,7 @@
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">ул. Кирова, 12 (ЛиЛия)</t>
+          <t xml:space="preserve">ул. Кирова, 12</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
@@ -4661,7 +4661,7 @@
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">ул. Кирова, 12 (ЛиЛия)</t>
+          <t xml:space="preserve">ул. Кирова, 12</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
@@ -4713,7 +4713,7 @@
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">ул. Кирова, 12 (ЛиЛия)</t>
+          <t xml:space="preserve">ул. Кирова, 12</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">

</xml_diff>